<commit_message>
feat: Nuevo modulo de Oportunidades V 17.2
</commit_message>
<xml_diff>
--- a/proyectos_diseno/BASES_DE_DATOS/Avance_Proyectos.xlsx
+++ b/proyectos_diseno/BASES_DE_DATOS/Avance_Proyectos.xlsx
@@ -11455,9 +11455,13 @@
         <v>5</v>
       </c>
       <c r="G324" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H324" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H324" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -11487,9 +11491,13 @@
         <v>5</v>
       </c>
       <c r="G325" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H325" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H325" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
@@ -11519,9 +11527,13 @@
         <v>15</v>
       </c>
       <c r="G326" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H326" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H326" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -11551,9 +11563,13 @@
         <v>5</v>
       </c>
       <c r="G327" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H327" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
@@ -11583,9 +11599,13 @@
         <v>10</v>
       </c>
       <c r="G328" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H328" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -11615,9 +11635,13 @@
         <v>10</v>
       </c>
       <c r="G329" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H329" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -11647,9 +11671,13 @@
         <v>10</v>
       </c>
       <c r="G330" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H330" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
@@ -11679,9 +11707,13 @@
         <v>2.5</v>
       </c>
       <c r="G331" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H331" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -11711,9 +11743,13 @@
         <v>10</v>
       </c>
       <c r="G332" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H332" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -11743,9 +11779,13 @@
         <v>7.5</v>
       </c>
       <c r="G333" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H333" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -11775,9 +11815,13 @@
         <v>5</v>
       </c>
       <c r="G334" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H334" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -11807,9 +11851,13 @@
         <v>10</v>
       </c>
       <c r="G335" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H335" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -11839,9 +11887,13 @@
         <v>5</v>
       </c>
       <c r="G336" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H336" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">

</xml_diff>

<commit_message>
test: ARchivs de prueba
</commit_message>
<xml_diff>
--- a/proyectos_diseno/BASES_DE_DATOS/Avance_Proyectos.xlsx
+++ b/proyectos_diseno/BASES_DE_DATOS/Avance_Proyectos.xlsx
@@ -4695,9 +4695,13 @@
         <v>5</v>
       </c>
       <c r="G122" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H122" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">

</xml_diff>